<commit_message>
Thêm tab sang kiện thay bọc
</commit_message>
<xml_diff>
--- a/cung_cap_dl/sl_mau.xlsx
+++ b/cung_cap_dl/sl_mau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Software\rubber-erp\cung_cap_dl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3319E7EA-58AC-482F-9E49-711C7BCEAE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC18342A-9BD9-4D3E-9D6F-F36FF453C6D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="17">
   <si>
     <t>Ngày</t>
   </si>
@@ -64,37 +64,19 @@
     <t>1A</t>
   </si>
   <si>
-    <t>1A2</t>
-  </si>
-  <si>
     <t>Đội</t>
   </si>
   <si>
-    <t>11A</t>
-  </si>
-  <si>
-    <t>11A2</t>
-  </si>
-  <si>
-    <t>13A</t>
-  </si>
-  <si>
-    <t>13A2</t>
-  </si>
-  <si>
-    <t>15A</t>
-  </si>
-  <si>
-    <t>18A</t>
-  </si>
-  <si>
-    <t>19A</t>
-  </si>
-  <si>
-    <t>22A</t>
-  </si>
-  <si>
-    <t>3A</t>
+    <t>16A</t>
+  </si>
+  <si>
+    <t>16A2</t>
+  </si>
+  <si>
+    <t>8A</t>
+  </si>
+  <si>
+    <t>10A</t>
   </si>
 </sst>
 </file>
@@ -459,7 +441,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>1</v>
@@ -542,7 +524,7 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
@@ -557,36 +539,36 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="3">
-        <v>2120</v>
+        <v>2090</v>
       </c>
       <c r="K3" s="1">
-        <v>55.16</v>
+        <v>56.42</v>
       </c>
       <c r="L3" s="4">
-        <v>1169.3900000000001</v>
+        <v>1179.18</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
       <c r="P3" s="1">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="Q3" s="1">
         <v>65</v>
       </c>
       <c r="R3" s="1">
-        <v>15.6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -595,36 +577,36 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="3">
-        <v>2530</v>
+        <v>1480</v>
       </c>
       <c r="K4" s="1">
-        <v>54.63</v>
+        <v>56.47</v>
       </c>
       <c r="L4" s="4">
-        <v>1382.14</v>
+        <v>835.76</v>
       </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="Q4" s="1">
         <v>65</v>
       </c>
       <c r="R4" s="1">
-        <v>21.45</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B5" s="1">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -633,30 +615,30 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="3">
-        <v>2210</v>
+        <v>1860</v>
       </c>
       <c r="K5" s="1">
-        <v>55.65</v>
+        <v>56.6</v>
       </c>
       <c r="L5" s="4">
-        <v>1229.8699999999999</v>
+        <v>1052.76</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="Q5" s="1">
         <v>65</v>
       </c>
       <c r="R5" s="1">
-        <v>14.3</v>
+        <v>17.55</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B6" s="1">
         <v>4</v>
@@ -671,36 +653,36 @@
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="3">
-        <v>1550</v>
+        <v>1910</v>
       </c>
       <c r="K6" s="1">
-        <v>54.33</v>
-      </c>
-      <c r="L6" s="1">
-        <v>842.12</v>
+        <v>56.41</v>
+      </c>
+      <c r="L6" s="4">
+        <v>1077.43</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="Q6" s="1">
         <v>65</v>
       </c>
       <c r="R6" s="1">
-        <v>16.25</v>
+        <v>26.65</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B7" s="1">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -709,36 +691,36 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="3">
-        <v>1850</v>
+        <v>1910</v>
       </c>
       <c r="K7" s="1">
-        <v>54.21</v>
+        <v>55.82</v>
       </c>
       <c r="L7" s="4">
-        <v>1002.89</v>
+        <v>1066.1600000000001</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="Q7" s="1">
         <v>65</v>
       </c>
       <c r="R7" s="1">
-        <v>15.6</v>
+        <v>25.35</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B8" s="1">
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -747,36 +729,36 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="3">
-        <v>1240</v>
+        <v>1900</v>
       </c>
       <c r="K8" s="1">
-        <v>55.1</v>
-      </c>
-      <c r="L8" s="1">
-        <v>683.24</v>
+        <v>55.56</v>
+      </c>
+      <c r="L8" s="4">
+        <v>1055.6400000000001</v>
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="Q8" s="1">
         <v>65</v>
       </c>
       <c r="R8" s="1">
-        <v>18.2</v>
+        <v>39.65</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B9" s="1">
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -785,36 +767,36 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="3">
-        <v>1080</v>
+        <v>1130</v>
       </c>
       <c r="K9" s="1">
-        <v>55.16</v>
+        <v>55.43</v>
       </c>
       <c r="L9" s="1">
-        <v>595.73</v>
+        <v>626.36</v>
       </c>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="Q9" s="1">
         <v>65</v>
       </c>
       <c r="R9" s="1">
-        <v>11.7</v>
+        <v>16.899999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B10" s="1">
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -823,36 +805,36 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="3">
-        <v>1190</v>
+        <v>2000</v>
       </c>
       <c r="K10" s="1">
-        <v>55.69</v>
-      </c>
-      <c r="L10" s="1">
-        <v>662.71</v>
+        <v>56.03</v>
+      </c>
+      <c r="L10" s="4">
+        <v>1120.5999999999999</v>
       </c>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="Q10" s="1">
         <v>65</v>
       </c>
       <c r="R10" s="1">
-        <v>19.5</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B11" s="1">
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -861,36 +843,36 @@
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="3">
-        <v>1840</v>
+        <v>2390</v>
       </c>
       <c r="K11" s="1">
-        <v>54.11</v>
-      </c>
-      <c r="L11" s="1">
-        <v>995.62</v>
+        <v>56.19</v>
+      </c>
+      <c r="L11" s="4">
+        <v>1342.94</v>
       </c>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="Q11" s="1">
         <v>65</v>
       </c>
       <c r="R11" s="1">
-        <v>20.8</v>
+        <v>41.6</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B12" s="1">
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -899,36 +881,36 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="3">
-        <v>1850</v>
+        <v>2370</v>
       </c>
       <c r="K12" s="1">
-        <v>54.52</v>
+        <v>56.13</v>
       </c>
       <c r="L12" s="4">
-        <v>1008.62</v>
+        <v>1330.28</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="Q12" s="1">
         <v>65</v>
       </c>
       <c r="R12" s="1">
-        <v>16.899999999999999</v>
+        <v>38.35</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B13" s="1">
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -937,36 +919,36 @@
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="3">
-        <v>1930</v>
+        <v>2100</v>
       </c>
       <c r="K13" s="1">
-        <v>55.6</v>
+        <v>55.74</v>
       </c>
       <c r="L13" s="4">
-        <v>1073.08</v>
+        <v>1170.54</v>
       </c>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="Q13" s="1">
         <v>65</v>
       </c>
       <c r="R13" s="1">
-        <v>18.2</v>
+        <v>31.85</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B14" s="1">
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -975,25 +957,25 @@
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="3">
-        <v>1870</v>
+        <v>1400</v>
       </c>
       <c r="K14" s="1">
-        <v>55.19</v>
+        <v>56.08</v>
       </c>
       <c r="L14" s="4">
-        <v>1032.05</v>
+        <v>785.12</v>
       </c>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="Q14" s="1">
         <v>65</v>
       </c>
       <c r="R14" s="1">
-        <v>16.899999999999999</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fix bug modun ISO
</commit_message>
<xml_diff>
--- a/cung_cap_dl/sl_mau.xlsx
+++ b/cung_cap_dl/sl_mau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Software\rubber-erp\cung_cap_dl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC18342A-9BD9-4D3E-9D6F-F36FF453C6D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A722B6-FA06-4A33-AFF9-36F3CD13A28A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="18">
   <si>
     <t>Ngày</t>
   </si>
@@ -70,13 +70,16 @@
     <t>16A</t>
   </si>
   <si>
-    <t>16A2</t>
+    <t>10A</t>
   </si>
   <si>
-    <t>8A</t>
+    <t>11A</t>
   </si>
   <si>
-    <t>10A</t>
+    <t>18A</t>
+  </si>
+  <si>
+    <t>19A</t>
   </si>
 </sst>
 </file>
@@ -429,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -524,13 +527,13 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -539,36 +542,36 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="3">
-        <v>2090</v>
+        <v>3960</v>
       </c>
       <c r="K3" s="1">
-        <v>56.42</v>
+        <v>55.45</v>
       </c>
       <c r="L3" s="4">
-        <v>1179.18</v>
+        <v>2195.8200000000002</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
       <c r="P3" s="1">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="Q3" s="1">
         <v>65</v>
       </c>
       <c r="R3" s="1">
-        <v>26</v>
+        <v>61.75</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -577,36 +580,36 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="3">
-        <v>1480</v>
+        <v>4150</v>
       </c>
       <c r="K4" s="1">
-        <v>56.47</v>
+        <v>55.65</v>
       </c>
       <c r="L4" s="4">
-        <v>835.76</v>
+        <v>2309.48</v>
       </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="Q4" s="1">
         <v>65</v>
       </c>
       <c r="R4" s="1">
-        <v>19.5</v>
+        <v>16.25</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B5" s="1">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -615,36 +618,36 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="3">
-        <v>1860</v>
+        <v>4030</v>
       </c>
       <c r="K5" s="1">
-        <v>56.6</v>
+        <v>54.87</v>
       </c>
       <c r="L5" s="4">
-        <v>1052.76</v>
+        <v>2211.2600000000002</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="Q5" s="1">
         <v>65</v>
       </c>
       <c r="R5" s="1">
-        <v>17.55</v>
+        <v>55.25</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B6" s="1">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -653,36 +656,36 @@
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="3">
-        <v>1910</v>
+        <v>3550</v>
       </c>
       <c r="K6" s="1">
-        <v>56.41</v>
+        <v>55.14</v>
       </c>
       <c r="L6" s="4">
-        <v>1077.43</v>
+        <v>1957.47</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Q6" s="1">
         <v>65</v>
       </c>
       <c r="R6" s="1">
-        <v>26.65</v>
+        <v>24.05</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B7" s="1">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -691,36 +694,36 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="3">
-        <v>1910</v>
+        <v>3660</v>
       </c>
       <c r="K7" s="1">
-        <v>55.82</v>
+        <v>55.26</v>
       </c>
       <c r="L7" s="4">
-        <v>1066.1600000000001</v>
+        <v>2022.52</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1">
-        <v>39</v>
+        <v>96</v>
       </c>
       <c r="Q7" s="1">
         <v>65</v>
       </c>
       <c r="R7" s="1">
-        <v>25.35</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B8" s="1">
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -729,36 +732,36 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="3">
-        <v>1900</v>
+        <v>3140</v>
       </c>
       <c r="K8" s="1">
-        <v>55.56</v>
+        <v>55.35</v>
       </c>
       <c r="L8" s="4">
-        <v>1055.6400000000001</v>
+        <v>1737.99</v>
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1">
-        <v>61</v>
+        <v>105</v>
       </c>
       <c r="Q8" s="1">
         <v>65</v>
       </c>
       <c r="R8" s="1">
-        <v>39.65</v>
+        <v>68.25</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B9" s="1">
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -767,36 +770,36 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="3">
-        <v>1130</v>
+        <v>2630</v>
       </c>
       <c r="K9" s="1">
-        <v>55.43</v>
-      </c>
-      <c r="L9" s="1">
-        <v>626.36</v>
+        <v>55.49</v>
+      </c>
+      <c r="L9" s="4">
+        <v>1459.39</v>
       </c>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1">
-        <v>26</v>
+        <v>78</v>
       </c>
       <c r="Q9" s="1">
         <v>65</v>
       </c>
       <c r="R9" s="1">
-        <v>16.899999999999999</v>
+        <v>50.7</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B10" s="1">
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -805,36 +808,36 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="3">
-        <v>2000</v>
+        <v>2880</v>
       </c>
       <c r="K10" s="1">
-        <v>56.03</v>
+        <v>54.63</v>
       </c>
       <c r="L10" s="4">
-        <v>1120.5999999999999</v>
+        <v>1573.34</v>
       </c>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="Q10" s="1">
         <v>65</v>
       </c>
       <c r="R10" s="1">
-        <v>35.1</v>
+        <v>74.75</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B11" s="1">
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -843,36 +846,36 @@
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="3">
-        <v>2390</v>
+        <v>2750</v>
       </c>
       <c r="K11" s="1">
-        <v>56.19</v>
+        <v>54.1</v>
       </c>
       <c r="L11" s="4">
-        <v>1342.94</v>
+        <v>1487.75</v>
       </c>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="Q11" s="1">
         <v>65</v>
       </c>
       <c r="R11" s="1">
-        <v>41.6</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B12" s="1">
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -881,36 +884,36 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="3">
-        <v>2370</v>
+        <v>3140</v>
       </c>
       <c r="K12" s="1">
-        <v>56.13</v>
+        <v>55.19</v>
       </c>
       <c r="L12" s="4">
-        <v>1330.28</v>
+        <v>1732.97</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="Q12" s="1">
         <v>65</v>
       </c>
       <c r="R12" s="1">
-        <v>38.35</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B13" s="1">
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -919,36 +922,36 @@
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="3">
-        <v>2100</v>
+        <v>2910</v>
       </c>
       <c r="K13" s="1">
-        <v>55.74</v>
+        <v>55.84</v>
       </c>
       <c r="L13" s="4">
-        <v>1170.54</v>
+        <v>1624.94</v>
       </c>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="Q13" s="1">
         <v>65</v>
       </c>
       <c r="R13" s="1">
-        <v>31.85</v>
+        <v>11.05</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <v>46162</v>
+        <v>46168</v>
       </c>
       <c r="B14" s="1">
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -957,25 +960,25 @@
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="3">
-        <v>1400</v>
+        <v>3510</v>
       </c>
       <c r="K14" s="1">
-        <v>56.08</v>
+        <v>54.82</v>
       </c>
       <c r="L14" s="4">
-        <v>785.12</v>
+        <v>1924.18</v>
       </c>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="Q14" s="1">
         <v>65</v>
       </c>
       <c r="R14" s="1">
-        <v>35.1</v>
+        <v>38.35</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
@@ -1050,7 +1053,7 @@
       <c r="I18" s="1"/>
       <c r="J18" s="3"/>
       <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
+      <c r="L18" s="4"/>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
@@ -1070,7 +1073,7 @@
       <c r="I19" s="1"/>
       <c r="J19" s="3"/>
       <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
+      <c r="L19" s="4"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
@@ -1090,7 +1093,7 @@
       <c r="I20" s="1"/>
       <c r="J20" s="3"/>
       <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
+      <c r="L20" s="4"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
@@ -1110,7 +1113,7 @@
       <c r="I21" s="1"/>
       <c r="J21" s="3"/>
       <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
+      <c r="L21" s="4"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
@@ -1130,7 +1133,7 @@
       <c r="I22" s="1"/>
       <c r="J22" s="3"/>
       <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
+      <c r="L22" s="4"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
@@ -1150,7 +1153,7 @@
       <c r="I23" s="1"/>
       <c r="J23" s="3"/>
       <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
+      <c r="L23" s="4"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
@@ -1170,7 +1173,7 @@
       <c r="I24" s="1"/>
       <c r="J24" s="3"/>
       <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
+      <c r="L24" s="4"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
@@ -1218,6 +1221,966 @@
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
     </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A27" s="2"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A28" s="2"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A29" s="2"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
+      <c r="R29" s="1"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A30" s="2"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A31" s="2"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="4"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A32" s="2"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A33" s="2"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A34" s="2"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A35" s="2"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="4"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+      <c r="P35" s="1"/>
+      <c r="Q35" s="1"/>
+      <c r="R35" s="1"/>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A36" s="2"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1"/>
+      <c r="P36" s="1"/>
+      <c r="Q36" s="1"/>
+      <c r="R36" s="1"/>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A37" s="2"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
+      <c r="P37" s="1"/>
+      <c r="Q37" s="1"/>
+      <c r="R37" s="1"/>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A38" s="2"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="4"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1"/>
+      <c r="P38" s="1"/>
+      <c r="Q38" s="1"/>
+      <c r="R38" s="1"/>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A39" s="2"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+      <c r="P39" s="1"/>
+      <c r="Q39" s="1"/>
+      <c r="R39" s="1"/>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A40" s="2"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="1"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="1"/>
+      <c r="N40" s="1"/>
+      <c r="O40" s="1"/>
+      <c r="P40" s="1"/>
+      <c r="Q40" s="1"/>
+      <c r="R40" s="1"/>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A41" s="2"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="1"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="1"/>
+      <c r="N41" s="1"/>
+      <c r="O41" s="1"/>
+      <c r="P41" s="1"/>
+      <c r="Q41" s="1"/>
+      <c r="R41" s="1"/>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A42" s="2"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="1"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="1"/>
+      <c r="N42" s="1"/>
+      <c r="O42" s="1"/>
+      <c r="P42" s="1"/>
+      <c r="Q42" s="1"/>
+      <c r="R42" s="1"/>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A43" s="2"/>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+      <c r="I43" s="1"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="1"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="1"/>
+      <c r="N43" s="1"/>
+      <c r="O43" s="1"/>
+      <c r="P43" s="1"/>
+      <c r="Q43" s="1"/>
+      <c r="R43" s="1"/>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A44" s="2"/>
+      <c r="B44" s="1"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="1"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+      <c r="O44" s="1"/>
+      <c r="P44" s="1"/>
+      <c r="Q44" s="1"/>
+      <c r="R44" s="1"/>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A45" s="2"/>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="1"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1"/>
+      <c r="O45" s="1"/>
+      <c r="P45" s="1"/>
+      <c r="Q45" s="1"/>
+      <c r="R45" s="1"/>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A46" s="2"/>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="1"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="1"/>
+      <c r="N46" s="1"/>
+      <c r="O46" s="1"/>
+      <c r="P46" s="1"/>
+      <c r="Q46" s="1"/>
+      <c r="R46" s="1"/>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A47" s="2"/>
+      <c r="B47" s="1"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="1"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1"/>
+      <c r="O47" s="1"/>
+      <c r="P47" s="1"/>
+      <c r="Q47" s="1"/>
+      <c r="R47" s="1"/>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A48" s="2"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="1"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="1"/>
+      <c r="N48" s="1"/>
+      <c r="O48" s="1"/>
+      <c r="P48" s="1"/>
+      <c r="Q48" s="1"/>
+      <c r="R48" s="1"/>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A49" s="2"/>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="1"/>
+      <c r="L49" s="4"/>
+      <c r="M49" s="1"/>
+      <c r="N49" s="1"/>
+      <c r="O49" s="1"/>
+      <c r="P49" s="1"/>
+      <c r="Q49" s="1"/>
+      <c r="R49" s="1"/>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A50" s="2"/>
+      <c r="B50" s="1"/>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="1"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="1"/>
+      <c r="N50" s="1"/>
+      <c r="O50" s="1"/>
+      <c r="P50" s="1"/>
+      <c r="Q50" s="1"/>
+      <c r="R50" s="1"/>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A51" s="2"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+      <c r="I51" s="1"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="1"/>
+      <c r="L51" s="4"/>
+      <c r="M51" s="1"/>
+      <c r="N51" s="1"/>
+      <c r="O51" s="1"/>
+      <c r="P51" s="1"/>
+      <c r="Q51" s="1"/>
+      <c r="R51" s="1"/>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A52" s="2"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="1"/>
+      <c r="L52" s="4"/>
+      <c r="M52" s="1"/>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1"/>
+      <c r="P52" s="1"/>
+      <c r="Q52" s="1"/>
+      <c r="R52" s="1"/>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A53" s="2"/>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1"/>
+      <c r="J53" s="3"/>
+      <c r="K53" s="1"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="1"/>
+      <c r="N53" s="1"/>
+      <c r="O53" s="1"/>
+      <c r="P53" s="1"/>
+      <c r="Q53" s="1"/>
+      <c r="R53" s="1"/>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A54" s="2"/>
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="1"/>
+      <c r="N54" s="1"/>
+      <c r="O54" s="1"/>
+      <c r="P54" s="1"/>
+      <c r="Q54" s="1"/>
+      <c r="R54" s="1"/>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A55" s="2"/>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1"/>
+      <c r="J55" s="3"/>
+      <c r="K55" s="1"/>
+      <c r="L55" s="4"/>
+      <c r="M55" s="1"/>
+      <c r="N55" s="1"/>
+      <c r="O55" s="1"/>
+      <c r="P55" s="1"/>
+      <c r="Q55" s="1"/>
+      <c r="R55" s="1"/>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A56" s="2"/>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1"/>
+      <c r="J56" s="3"/>
+      <c r="K56" s="1"/>
+      <c r="L56" s="4"/>
+      <c r="M56" s="1"/>
+      <c r="N56" s="1"/>
+      <c r="O56" s="1"/>
+      <c r="P56" s="1"/>
+      <c r="Q56" s="1"/>
+      <c r="R56" s="1"/>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A57" s="2"/>
+      <c r="B57" s="1"/>
+      <c r="C57" s="1"/>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+      <c r="I57" s="1"/>
+      <c r="J57" s="3"/>
+      <c r="K57" s="1"/>
+      <c r="L57" s="4"/>
+      <c r="M57" s="1"/>
+      <c r="N57" s="1"/>
+      <c r="O57" s="1"/>
+      <c r="P57" s="1"/>
+      <c r="Q57" s="1"/>
+      <c r="R57" s="1"/>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A58" s="2"/>
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+      <c r="J58" s="3"/>
+      <c r="K58" s="1"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="1"/>
+      <c r="N58" s="1"/>
+      <c r="O58" s="1"/>
+      <c r="P58" s="1"/>
+      <c r="Q58" s="1"/>
+      <c r="R58" s="1"/>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A59" s="2"/>
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+      <c r="I59" s="1"/>
+      <c r="J59" s="3"/>
+      <c r="K59" s="1"/>
+      <c r="L59" s="4"/>
+      <c r="M59" s="1"/>
+      <c r="N59" s="1"/>
+      <c r="O59" s="1"/>
+      <c r="P59" s="1"/>
+      <c r="Q59" s="1"/>
+      <c r="R59" s="1"/>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A60" s="2"/>
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1"/>
+      <c r="J60" s="3"/>
+      <c r="K60" s="1"/>
+      <c r="L60" s="4"/>
+      <c r="M60" s="1"/>
+      <c r="N60" s="1"/>
+      <c r="O60" s="1"/>
+      <c r="P60" s="1"/>
+      <c r="Q60" s="1"/>
+      <c r="R60" s="1"/>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A61" s="2"/>
+      <c r="B61" s="1"/>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
+      <c r="I61" s="1"/>
+      <c r="J61" s="3"/>
+      <c r="K61" s="1"/>
+      <c r="L61" s="4"/>
+      <c r="M61" s="1"/>
+      <c r="N61" s="1"/>
+      <c r="O61" s="1"/>
+      <c r="P61" s="1"/>
+      <c r="Q61" s="1"/>
+      <c r="R61" s="1"/>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A62" s="2"/>
+      <c r="B62" s="1"/>
+      <c r="C62" s="1"/>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+      <c r="I62" s="1"/>
+      <c r="J62" s="3"/>
+      <c r="K62" s="1"/>
+      <c r="L62" s="4"/>
+      <c r="M62" s="1"/>
+      <c r="N62" s="1"/>
+      <c r="O62" s="1"/>
+      <c r="P62" s="1"/>
+      <c r="Q62" s="1"/>
+      <c r="R62" s="1"/>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A63" s="2"/>
+      <c r="B63" s="1"/>
+      <c r="C63" s="1"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+      <c r="I63" s="1"/>
+      <c r="J63" s="3"/>
+      <c r="K63" s="1"/>
+      <c r="L63" s="4"/>
+      <c r="M63" s="1"/>
+      <c r="N63" s="1"/>
+      <c r="O63" s="1"/>
+      <c r="P63" s="1"/>
+      <c r="Q63" s="1"/>
+      <c r="R63" s="1"/>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A64" s="2"/>
+      <c r="B64" s="1"/>
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+      <c r="I64" s="1"/>
+      <c r="J64" s="3"/>
+      <c r="K64" s="1"/>
+      <c r="L64" s="4"/>
+      <c r="M64" s="1"/>
+      <c r="N64" s="1"/>
+      <c r="O64" s="1"/>
+      <c r="P64" s="1"/>
+      <c r="Q64" s="1"/>
+      <c r="R64" s="1"/>
+    </row>
+    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A65" s="2"/>
+      <c r="B65" s="1"/>
+      <c r="C65" s="1"/>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1"/>
+      <c r="I65" s="1"/>
+      <c r="J65" s="3"/>
+      <c r="K65" s="1"/>
+      <c r="L65" s="4"/>
+      <c r="M65" s="1"/>
+      <c r="N65" s="1"/>
+      <c r="O65" s="1"/>
+      <c r="P65" s="1"/>
+      <c r="Q65" s="1"/>
+      <c r="R65" s="1"/>
+    </row>
+    <row r="66" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A66" s="2"/>
+      <c r="B66" s="1"/>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+      <c r="I66" s="1"/>
+      <c r="J66" s="3"/>
+      <c r="K66" s="1"/>
+      <c r="L66" s="4"/>
+      <c r="M66" s="1"/>
+      <c r="N66" s="1"/>
+      <c r="O66" s="1"/>
+      <c r="P66" s="1"/>
+      <c r="Q66" s="1"/>
+      <c r="R66" s="1"/>
+    </row>
+    <row r="67" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A67" s="2"/>
+      <c r="B67" s="1"/>
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
+      <c r="H67" s="1"/>
+      <c r="I67" s="1"/>
+      <c r="J67" s="3"/>
+      <c r="K67" s="1"/>
+      <c r="L67" s="4"/>
+      <c r="M67" s="1"/>
+      <c r="N67" s="1"/>
+      <c r="O67" s="1"/>
+      <c r="P67" s="1"/>
+      <c r="Q67" s="1"/>
+      <c r="R67" s="1"/>
+    </row>
+    <row r="68" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A68" s="2"/>
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+      <c r="I68" s="1"/>
+      <c r="J68" s="3"/>
+      <c r="K68" s="1"/>
+      <c r="L68" s="4"/>
+      <c r="M68" s="1"/>
+      <c r="N68" s="1"/>
+      <c r="O68" s="1"/>
+      <c r="P68" s="1"/>
+      <c r="Q68" s="1"/>
+      <c r="R68" s="1"/>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A69" s="2"/>
+      <c r="B69" s="1"/>
+      <c r="C69" s="1"/>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+      <c r="I69" s="1"/>
+      <c r="J69" s="3"/>
+      <c r="K69" s="1"/>
+      <c r="L69" s="4"/>
+      <c r="M69" s="1"/>
+      <c r="N69" s="1"/>
+      <c r="O69" s="1"/>
+      <c r="P69" s="1"/>
+      <c r="Q69" s="1"/>
+      <c r="R69" s="1"/>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A70" s="2"/>
+      <c r="B70" s="1"/>
+      <c r="C70" s="1"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="1"/>
+      <c r="J70" s="3"/>
+      <c r="K70" s="1"/>
+      <c r="L70" s="4"/>
+      <c r="M70" s="1"/>
+      <c r="N70" s="1"/>
+      <c r="O70" s="1"/>
+      <c r="P70" s="1"/>
+      <c r="Q70" s="1"/>
+      <c r="R70" s="1"/>
+    </row>
+    <row r="71" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A71" s="2"/>
+      <c r="B71" s="1"/>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+      <c r="I71" s="1"/>
+      <c r="J71" s="3"/>
+      <c r="K71" s="1"/>
+      <c r="L71" s="4"/>
+      <c r="M71" s="1"/>
+      <c r="N71" s="1"/>
+      <c r="O71" s="1"/>
+      <c r="P71" s="1"/>
+      <c r="Q71" s="1"/>
+      <c r="R71" s="1"/>
+    </row>
+    <row r="72" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A72" s="2"/>
+      <c r="B72" s="1"/>
+      <c r="C72" s="1"/>
+      <c r="D72" s="1"/>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1"/>
+      <c r="G72" s="1"/>
+      <c r="H72" s="1"/>
+      <c r="I72" s="1"/>
+      <c r="J72" s="3"/>
+      <c r="K72" s="1"/>
+      <c r="L72" s="4"/>
+      <c r="M72" s="1"/>
+      <c r="N72" s="1"/>
+      <c r="O72" s="1"/>
+      <c r="P72" s="1"/>
+      <c r="Q72" s="1"/>
+      <c r="R72" s="1"/>
+    </row>
+    <row r="73" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A73" s="2"/>
+      <c r="B73" s="1"/>
+      <c r="C73" s="1"/>
+      <c r="D73" s="1"/>
+      <c r="E73" s="1"/>
+      <c r="F73" s="1"/>
+      <c r="G73" s="1"/>
+      <c r="H73" s="1"/>
+      <c r="I73" s="1"/>
+      <c r="J73" s="3"/>
+      <c r="K73" s="1"/>
+      <c r="L73" s="4"/>
+      <c r="M73" s="1"/>
+      <c r="N73" s="1"/>
+      <c r="O73" s="1"/>
+      <c r="P73" s="1"/>
+      <c r="Q73" s="1"/>
+      <c r="R73" s="1"/>
+    </row>
+    <row r="74" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A74" s="2"/>
+      <c r="B74" s="1"/>
+      <c r="C74" s="1"/>
+      <c r="D74" s="1"/>
+      <c r="E74" s="1"/>
+      <c r="F74" s="1"/>
+      <c r="G74" s="1"/>
+      <c r="H74" s="1"/>
+      <c r="I74" s="1"/>
+      <c r="J74" s="3"/>
+      <c r="K74" s="1"/>
+      <c r="L74" s="4"/>
+      <c r="M74" s="1"/>
+      <c r="N74" s="1"/>
+      <c r="O74" s="1"/>
+      <c r="P74" s="1"/>
+      <c r="Q74" s="1"/>
+      <c r="R74" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>